<commit_message>
feat: discord webhook integration for paper broker alerts
</commit_message>
<xml_diff>
--- a/reports/paper_trading_performance.xlsx
+++ b/reports/paper_trading_performance.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="26">
   <si>
     <t>timestamp</t>
   </si>
@@ -460,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1225,6 +1225,120 @@
       </c>
       <c r="L20">
         <v>12.67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="3">
+        <v>46186.16352501582</v>
+      </c>
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21">
+        <v>0.072474</v>
+      </c>
+      <c r="E21">
+        <v>7434.58</v>
+      </c>
+      <c r="F21">
+        <v>538.8099999999999</v>
+      </c>
+      <c r="G21">
+        <v>0.27</v>
+      </c>
+      <c r="H21">
+        <v>9961.396561979996</v>
+      </c>
+      <c r="I21">
+        <v>15.29372664624316</v>
+      </c>
+      <c r="J21">
+        <v>-53.89716466624392</v>
+      </c>
+      <c r="K21">
+        <v>-38.60343802000077</v>
+      </c>
+      <c r="L21">
+        <v>12.94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="3">
+        <v>46186.16824081628</v>
+      </c>
+      <c r="B22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22">
+        <v>0.067011</v>
+      </c>
+      <c r="E22">
+        <v>7434.58</v>
+      </c>
+      <c r="F22">
+        <v>498.2</v>
+      </c>
+      <c r="G22">
+        <v>0.25</v>
+      </c>
+      <c r="H22">
+        <v>9961.395202359996</v>
+      </c>
+      <c r="I22">
+        <v>15.29236702624303</v>
+      </c>
+      <c r="J22">
+        <v>-53.89716466624392</v>
+      </c>
+      <c r="K22">
+        <v>-38.6047976400009</v>
+      </c>
+      <c r="L22">
+        <v>13.19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="3">
+        <v>46186.17084117234</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23">
+        <v>0.002659</v>
+      </c>
+      <c r="E23">
+        <v>7427.14</v>
+      </c>
+      <c r="F23">
+        <v>19.75</v>
+      </c>
+      <c r="G23">
+        <v>0.01</v>
+      </c>
+      <c r="H23">
+        <v>9958.215524619996</v>
+      </c>
+      <c r="I23">
+        <v>12.03613011580455</v>
+      </c>
+      <c r="J23">
+        <v>-53.8206054958056</v>
+      </c>
+      <c r="K23">
+        <v>-41.78447538000105</v>
+      </c>
+      <c r="L23">
+        <v>13.2</v>
       </c>
     </row>
   </sheetData>
@@ -1254,7 +1368,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1262,7 +1376,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1270,7 +1384,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1278,7 +1392,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>12.67</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1286,7 +1400,7 @@
         <v>21</v>
       </c>
       <c r="B6">
-        <v>25353.91</v>
+        <v>26410.67</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1294,7 +1408,7 @@
         <v>22</v>
       </c>
       <c r="B7">
-        <v>-53.9</v>
+        <v>-53.82</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1302,7 +1416,7 @@
         <v>23</v>
       </c>
       <c r="B8">
-        <v>12.79</v>
+        <v>12.04</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1310,7 +1424,7 @@
         <v>24</v>
       </c>
       <c r="B9">
-        <v>-41.11</v>
+        <v>-41.78</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1318,7 +1432,7 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>9958.889999999999</v>
+        <v>9958.219999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: updates to paper broker, build report, and fetch market data
</commit_message>
<xml_diff>
--- a/reports/paper_trading_performance.xlsx
+++ b/reports/paper_trading_performance.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="26">
   <si>
     <t>timestamp</t>
   </si>
@@ -460,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1339,6 +1339,44 @@
       </c>
       <c r="L23">
         <v>13.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="3">
+        <v>46186.18980320596</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24">
+        <v>0.00536</v>
+      </c>
+      <c r="E24">
+        <v>7434.58</v>
+      </c>
+      <c r="F24">
+        <v>39.85</v>
+      </c>
+      <c r="G24">
+        <v>0.02</v>
+      </c>
+      <c r="H24">
+        <v>9961.376002939996</v>
+      </c>
+      <c r="I24">
+        <v>15.19660843580459</v>
+      </c>
+      <c r="J24">
+        <v>-53.8206054958056</v>
+      </c>
+      <c r="K24">
+        <v>-38.62399706000101</v>
+      </c>
+      <c r="L24">
+        <v>13.22</v>
       </c>
     </row>
   </sheetData>
@@ -1368,7 +1406,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1376,7 +1414,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1392,7 +1430,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>13.2</v>
+        <v>13.22</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1400,7 +1438,7 @@
         <v>21</v>
       </c>
       <c r="B6">
-        <v>26410.67</v>
+        <v>26450.52</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1416,7 +1454,7 @@
         <v>23</v>
       </c>
       <c r="B8">
-        <v>12.04</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1424,7 +1462,7 @@
         <v>24</v>
       </c>
       <c r="B9">
-        <v>-41.78</v>
+        <v>-38.62</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1432,7 +1470,7 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>9958.219999999999</v>
+        <v>9961.379999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: simplify to v5.3.0 single LLM architecture and remove MoE echo chamber
</commit_message>
<xml_diff>
--- a/reports/paper_trading_performance.xlsx
+++ b/reports/paper_trading_performance.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="27">
   <si>
     <t>timestamp</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>SPX</t>
+  </si>
+  <si>
+    <t>Gold</t>
   </si>
   <si>
     <t>Metric</t>
@@ -460,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1377,6 +1380,82 @@
       </c>
       <c r="L24">
         <v>13.22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="3">
+        <v>46186.19893202635</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25">
+        <v>0.251223</v>
+      </c>
+      <c r="E25">
+        <v>4242.02</v>
+      </c>
+      <c r="F25">
+        <v>1065.69</v>
+      </c>
+      <c r="G25">
+        <v>0.53</v>
+      </c>
+      <c r="H25">
+        <v>9961.378993399996</v>
+      </c>
+      <c r="I25">
+        <v>15.19959889580446</v>
+      </c>
+      <c r="J25">
+        <v>-53.8206054958056</v>
+      </c>
+      <c r="K25">
+        <v>-38.62100660000115</v>
+      </c>
+      <c r="L25">
+        <v>13.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="3">
+        <v>46186.20421433327</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26">
+        <v>0.083158</v>
+      </c>
+      <c r="E26">
+        <v>7427.14</v>
+      </c>
+      <c r="F26">
+        <v>617.63</v>
+      </c>
+      <c r="G26">
+        <v>0.31</v>
+      </c>
+      <c r="H26">
+        <v>9958.181877359995</v>
+      </c>
+      <c r="I26">
+        <v>9.680063660558744</v>
+      </c>
+      <c r="J26">
+        <v>-51.49818630055986</v>
+      </c>
+      <c r="K26">
+        <v>-41.81812264000111</v>
+      </c>
+      <c r="L26">
+        <v>14.06</v>
       </c>
     </row>
   </sheetData>
@@ -1395,82 +1474,82 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5">
-        <v>13.22</v>
+        <v>14.06</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6">
-        <v>26450.52</v>
+        <v>28133.84</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7">
-        <v>-53.82</v>
+        <v>-51.5</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8">
-        <v>15.2</v>
+        <v>9.68</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9">
-        <v>-38.62</v>
+        <v>-41.82</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10">
-        <v>9961.379999999999</v>
+        <v>9958.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: continuous compounding simulator and v5.3.2 docs upgrade
</commit_message>
<xml_diff>
--- a/reports/paper_trading_performance.xlsx
+++ b/reports/paper_trading_performance.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="27">
   <si>
     <t>timestamp</t>
   </si>
@@ -463,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
@@ -1456,6 +1456,82 @@
       </c>
       <c r="L26">
         <v>14.06</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="3">
+        <v>46186.5862034704</v>
+      </c>
+      <c r="B27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27">
+        <v>0.109921</v>
+      </c>
+      <c r="E27">
+        <v>7427.14</v>
+      </c>
+      <c r="F27">
+        <v>816.4</v>
+      </c>
+      <c r="G27">
+        <v>0.41</v>
+      </c>
+      <c r="H27">
+        <v>9958.183221419997</v>
+      </c>
+      <c r="I27">
+        <v>6.615357426412629</v>
+      </c>
+      <c r="J27">
+        <v>-48.43213600641379</v>
+      </c>
+      <c r="K27">
+        <v>-41.81677858000116</v>
+      </c>
+      <c r="L27">
+        <v>14.47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="3">
+        <v>46186.58621225939</v>
+      </c>
+      <c r="B28" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28">
+        <v>0.084497</v>
+      </c>
+      <c r="E28">
+        <v>4237.78</v>
+      </c>
+      <c r="F28">
+        <v>358.08</v>
+      </c>
+      <c r="G28">
+        <v>0.18</v>
+      </c>
+      <c r="H28">
+        <v>9957.118339239996</v>
+      </c>
+      <c r="I28">
+        <v>5.907433367285421</v>
+      </c>
+      <c r="J28">
+        <v>-48.78909412728657</v>
+      </c>
+      <c r="K28">
+        <v>-42.88166076000115</v>
+      </c>
+      <c r="L28">
+        <v>14.65</v>
       </c>
     </row>
   </sheetData>
@@ -1485,7 +1561,7 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1501,7 +1577,7 @@
         <v>20</v>
       </c>
       <c r="B4">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1509,7 +1585,7 @@
         <v>21</v>
       </c>
       <c r="B5">
-        <v>14.06</v>
+        <v>14.65</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1517,7 +1593,7 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>28133.84</v>
+        <v>29308.32</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1525,7 +1601,7 @@
         <v>23</v>
       </c>
       <c r="B7">
-        <v>-51.5</v>
+        <v>-48.79</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1533,7 +1609,7 @@
         <v>24</v>
       </c>
       <c r="B8">
-        <v>9.68</v>
+        <v>5.91</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1541,7 +1617,7 @@
         <v>25</v>
       </c>
       <c r="B9">
-        <v>-41.82</v>
+        <v>-42.88</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1549,7 +1625,7 @@
         <v>26</v>
       </c>
       <c r="B10">
-        <v>9958.18</v>
+        <v>9957.120000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>